<commit_message>
fix: phantom drive — correct D7/OK1 orientation, 80V opto, drop C16
- D7 zener was reversed (Vgs clamped at -0.7V, FET never switched);
  cathode now to V_FILT, anode to Q1_GATE.
- OK1 optocoupler C/E were swapped in the symbol (pin3/pin4), exceeding
  its 6V emitter-collector reverse rating on the PoE rail and holding
  phantom on in both switch positions; collector->R13/gate, emitter->PGND.
- OK1 -> TLP291 (80V Vceo), SOP-4 1.27mm; LTV-817's 35V was under-rated
  for the 46-57V PoE rail.
- Remove C16 (10uF): it sat on the tapped bus and broke 802.3 PoE
  detection (>0.15uF), which blocked cold-start with the tap connected.
- Regenerate fab set (gerbers, drills, CPL, BOM) for the above.
</commit_message>
<xml_diff>
--- a/fab/scramble_hat-BOM.xlsx
+++ b/fab/scramble_hat-BOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,7 +485,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Optocoupler</t>
+          <t>Optocoupler 80V</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -495,12 +495,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SO-4</t>
+          <t>SOP-4-1.27mm</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>C114603</t>
+          <t>C393895</t>
         </is>
       </c>
     </row>
@@ -771,136 +771,129 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10uF 100V X7S</t>
+          <t>100nF 100V X7R</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C17</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1210</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>C22380050</t>
+          <t>C89258</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>100nF 100V X7R</t>
+          <t>1uF 100V X7R</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C18</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>1206</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>C89258</t>
+          <t>C13832</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1uF 100V X7R</t>
+          <t>2.2uF 10V X5R</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>C22</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1206</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C13832</t>
+          <t>C107369</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2.2uF 10V X5R</t>
+          <t>10k 1%</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>C22</t>
+          <t>R1,R2,R3,R4</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>0402</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>C107369</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10k 1%</t>
+          <t>6.81k 1%</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>R1,R2,R3,R4</t>
+          <t>R5,R6</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0402</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
+          <t>0805</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>6.81k 1%</t>
+          <t>2.2k 1%</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>R5,R6</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
+          <t>0402</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2.2k 1%</t>
+          <t>33R 1%</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R9,R10</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -908,17 +901,16 @@
           <t>0402</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>33R 1%</t>
+          <t>100k 1%</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>R9,R10</t>
+          <t>R11,R13</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -926,17 +918,16 @@
           <t>0402</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>100k 1%</t>
+          <t>1k 1%</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>R11,R13</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -944,83 +935,63 @@
           <t>0402</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1k 1%</t>
+          <t>33k 1%</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>R16</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0402</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
+          <t>0805</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>33k 1%</t>
+          <t>1x7 female socket, 8.5mm</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>R16</t>
+          <t>J3,J4</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
+          <t>PinSocket_1x07_2.54mm TH</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>C2832270</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1x7 female socket, 8.5mm</t>
+          <t>SPDT slide switch (phantom on/off)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>J3,J4</t>
+          <t>SW1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PinSocket_1x07_2.54mm TH</t>
+          <t>SW_Slide_SS-12D00-G3 TH</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
-        <is>
-          <t>C2832270</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>SPDT slide switch (phantom on/off)</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>SW1</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>SW_Slide_SS-12D00-G3 TH</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
         <is>
           <t>C22355741</t>
         </is>

</xml_diff>

<commit_message>
fab: production prep — white/brighter status LED, C19 assembled, live BOM prices
- D8 red -> white: KT-0805W (C34499, Basic, in stock); old Kingbright
  KP-2012EC (C598272) was out of stock.
- R16 33k -> 15k, 1/4W AC0805 (C20142753) — ~2x brighter phantom-present
  LED (~3mA); resistor dissipates ~193mW at the 57V PoE max.
- C19 -> JEC JY222M2FY5VS7LE (C389727, Y2 300VAC, same 7.5mm land, in
  stock) moved onto JLCPCB THT assembly (off the hand-solder list).
- exclude_from_pos_files on J1/J2/J5 so placement/CPL leaves the
  hand-soldered parts (jacks + PoE header) to hand assembly.
- BOM: added J6, filled all resistor LCSC#s, refreshed unit prices to
  live qty-10 LCSC, corrected the D1/D2 entry.
- Regenerated gerbers/drills/BOM (csv+xlsx) with J6.
- Removed stale kicad-cli CPL — generate placement with the jlcpcb-tools
  plugin (set U1/QFN +270deg) and verify in JLCPCB preview before order.
</commit_message>
<xml_diff>
--- a/fab/scramble_hat-BOM.xlsx
+++ b/fab/scramble_hat-BOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>D1,D2</t>
+          <t>D1, D2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -595,7 +595,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LED, red</t>
+          <t>LED, white</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>C598272</t>
+          <t>C34499</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>C1,C3,C4</t>
+          <t>C1, C3, C4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>C2,C5,C7,C8,C9,C12,C13,C20,C21</t>
+          <t>C2, C5, C7, C8, C9, C12, C13, C20, C21</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>C10,C11</t>
+          <t>C10, C11</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>C14,C15</t>
+          <t>C14, C15</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -815,183 +815,262 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2.2uF 10V X5R</t>
+          <t>2.2nF Y2 250VAC</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>C22</t>
+          <t>C19</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>Disc TH</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C107369</t>
+          <t>C389727</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10k 1%</t>
+          <t>2.2uF 10V X5R</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R1,R2,R3,R4</t>
+          <t>C22</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>0402</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>C107369</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>6.81k 1%</t>
+          <t>10k 1%</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>R5,R6</t>
+          <t>R1, R2, R3, R4</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0402</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>C25744</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2.2k 1%</t>
+          <t>6.81k 1%</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R5, R6</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>C3025619</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>33R 1%</t>
+          <t>2.2k 1%</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>R9,R10</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>0402</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>C25879</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>100k 1%</t>
+          <t>33R 1%</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>R11,R13</t>
+          <t>R9, R10</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>0402</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>C25105</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1k 1%</t>
+          <t>100k 1%</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>R11, R13</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>0402</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>C25741</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>33k 1%</t>
+          <t>1k 1%</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>R16</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0402</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>C11702</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1x7 female socket, 8.5mm</t>
+          <t>15k 1% 1/4W</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>J3,J4</t>
+          <t>R16</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PinSocket_1x07_2.54mm TH</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>C2832270</t>
+          <t>C20142753</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>1x7 female socket, 8.5mm</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>J3, J4</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>PinSocket_1x07_2.54mm TH</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>C2832270</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1x4 pin header</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>J6</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>PinHeader_1x04_2.54mm TH</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>C124378</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>SPDT slide switch (phantom on/off)</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>SW1</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>SW_Slide_SS-12D00-G3 TH</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>C22355741</t>
         </is>

</xml_diff>

<commit_message>
fab: resolve JLCPCB short-supply flags (OK1, C19, R1-R4)
JLC flagged three parts short at qty-10; sourced in-stock fixes:

- OK1: TLP291 (C393895) -> Everlight EL3H7(C)(TA)-G (C92243). Same SOP-4 1.27mm land + opto pinout, 80V Vceo -> pure BOM swap, no layout change.
- C19: 2.2nF Y2 cap moved off the JLC line to hand-solder (every 7.5mm Y2 is thin at LCSC). Added exclude_from_pos_files in the PCB; BOM references Murata DE2E3SA222MA3BT02F for user sourcing.
- R1-R4: C25744 (UNI-ROYAL 0402WGF1002TCE, out of stock) was mislabeled with a Yageo MPN; corrected to the matching Yageo C60490 (10k 0402 1%, in stock).

Regenerated fab BOM (28 assembled parts) and CPL (48 placements; C19 now excluded alongside J1/J2/J5/R14). Gerbers unchanged.
</commit_message>
<xml_diff>
--- a/fab/scramble_hat-BOM.xlsx
+++ b/fab/scramble_hat-BOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,7 +500,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>C393895</t>
+          <t>C92243</t>
         </is>
       </c>
     </row>
@@ -815,34 +815,34 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2.2nF Y2 250VAC</t>
+          <t>2.2uF 10V X5R</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>C19</t>
+          <t>C22</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Disc TH</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C389727</t>
+          <t>C107369</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2.2uF 10V X5R</t>
+          <t>10k 1%</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>C22</t>
+          <t>R1, R2, R3, R4</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -852,63 +852,63 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>C107369</t>
+          <t>C60490</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10k 1%</t>
+          <t>6.81k 1%</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>R1, R2, R3, R4</t>
+          <t>R5, R6</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>C25744</t>
+          <t>C3025619</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>6.81k 1%</t>
+          <t>2.2k 1%</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>R5, R6</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>C3025619</t>
+          <t>C25879</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2.2k 1%</t>
+          <t>33R 1%</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R9, R10</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -918,19 +918,19 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>C25879</t>
+          <t>C25105</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>33R 1%</t>
+          <t>100k 1%</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>R9, R10</t>
+          <t>R11, R13</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -940,19 +940,19 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>C25105</t>
+          <t>C25741</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>100k 1%</t>
+          <t>1k 1%</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>R11, R13</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -962,115 +962,93 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>C25741</t>
+          <t>C11702</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1k 1%</t>
+          <t>15k 1% 1/4W</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>R16</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>C11702</t>
+          <t>C20142753</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>15k 1% 1/4W</t>
+          <t>1x7 female socket, 8.5mm</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>R16</t>
+          <t>J3, J4</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>PinSocket_1x07_2.54mm TH</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>C20142753</t>
+          <t>C2832270</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1x7 female socket, 8.5mm</t>
+          <t>1x4 pin header</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>J3, J4</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PinSocket_1x07_2.54mm TH</t>
+          <t>PinHeader_1x04_2.54mm TH</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>C2832270</t>
+          <t>C124378</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1x4 pin header</t>
+          <t>SPDT slide switch (phantom on/off)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>SW1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PinHeader_1x04_2.54mm TH</t>
+          <t>SW_Slide_SS-12D00-G3 TH</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
-        <is>
-          <t>C124378</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>SPDT slide switch (phantom on/off)</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>SW1</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>SW_Slide_SS-12D00-G3 TH</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
         <is>
           <t>C22355741</t>
         </is>

</xml_diff>

<commit_message>
pcb: place + route guitar input; regen fab
Layout for the guitar-input rev (U3 buffer, U4 mux, D9 tip ESD,
R19-R26/C23-C29, D1/D2 now SOD-323). Verified: DRC 0 errors /
0 unconnected, schematic sync clean (75 comps / 61 nets both sides).

Post-layout fixes:
- restore exclude_from_pos_files on C19/J1/J2/J5 (wiped again by
  re-layout; CPL correctly excludes C19,J1,J2,J5,R14)
- point D9 at the project-local 3D model (stock lib ships none)
- remove stale OK1_LED_A routing left from the mis-wired-label detour
  (1 via + 10 segments, all dangling; net verified intact throughout)

fab/ regenerated: gerbers/drills/zip, BOM 34 assembled, CPL 70 placed.
Order-time checks in the JLCPCB preview: U1 QFN (+270) first, then U4
TSSOP-16 (no rotation pattern) and K1/K2 SOP-4 (-90). D1/D2/D9 are
bidirectional two-terminal parts - rotation is not a concern.
</commit_message>
<xml_diff>
--- a/fab/scramble_hat-BOM.xlsx
+++ b/fab/scramble_hat-BOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,7 +529,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ESD array, 4-line</t>
+          <t>ESD diode, 3.3V bidir</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -539,12 +539,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SOT-353</t>
+          <t>SOD-323</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>C70500</t>
+          <t>C316020</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>C1, C3, C4</t>
+          <t>C1, C3, C4, C27, C28, C29</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>C2, C5, C7, C8, C9, C12, C13, C20, C21</t>
+          <t>C2, C5, C7, C8, C9, C12, C13, C20, C21, C23, C24, C25, C26</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R1, R2, R3, R4</t>
+          <t>R1, R2, R3, R4, R25</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R7, R20</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>R9, R10</t>
+          <t>R9, R10, R24</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -930,7 +930,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>R11, R13</t>
+          <t>R11, R13, R19, R22, R23</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1095,6 +1095,94 @@
       <c r="D31" t="inlineStr">
         <is>
           <t>C114877</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Op-amp Hi-Z buffer (RRIO CMOS)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>U3</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>SOT-23-5</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>C398358</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Analog switch triple SPDT</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>U4</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>TSSOP-16</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>C5648</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>1M 1%</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>R21, R26</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>0402</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>C26083</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ESD diode bidir 5.5V</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>X1-SON-2 0.6x1.0mm</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>C48260</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sch+pcb: dual-host mezzanine pinout (ESP32-P4 + Pico) — I2C to J3.1/2, BCLK/LRCK adjacent, MCLK/DET on J4.6/7, new R28 MCLK series link; regen fab + docs; add pinout graphic
</commit_message>
<xml_diff>
--- a/fab/scramble_hat-BOM.xlsx
+++ b/fab/scramble_hat-BOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,7 +500,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>C92243</t>
+          <t>C17549577</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C17, C30</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>C25879</t>
+          <t>C144773</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>C25105</t>
+          <t>C138002</t>
         </is>
       </c>
     </row>
@@ -940,7 +940,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>C25741</t>
+          <t>C60491</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>C11702</t>
+          <t>C106235</t>
         </is>
       </c>
     </row>
@@ -1013,174 +1013,152 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1x4 pin header</t>
+          <t>0R jumper 0805</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>R28</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PinHeader_1x04_2.54mm TH</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>C124378</t>
+          <t>C17477</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SPDT slide switch (phantom on/off)</t>
+          <t>PhotoMOS SSR 400V (tap disconnect)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SW1</t>
+          <t>K1, K2</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SW_Slide_SS-12D00-G3 TH</t>
+          <t>SOP-4 3.8x4.1mm</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>C22355741</t>
+          <t>C2890344</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PhotoMOS SSR 400V (tap disconnect)</t>
+          <t>470R 1% (PhotoMOS LED limit)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>K1, K2</t>
+          <t>R17, R18</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SOP-4 3.8x4.1mm</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>C2890344</t>
+          <t>C114877</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>470R 1% (PhotoMOS LED limit)</t>
+          <t>Op-amp Hi-Z buffer (RRIO CMOS)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>R17, R18</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>SOT-23-5</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>C114877</t>
+          <t>C398358</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Op-amp Hi-Z buffer (RRIO CMOS)</t>
+          <t>Analog switch triple SPDT</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>U4</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
+          <t>TSSOP-16</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>C398358</t>
+          <t>C5648</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Analog switch triple SPDT</t>
+          <t>1M 1%</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>U4</t>
+          <t>R21, R26</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>TSSOP-16</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>C5648</t>
+          <t>C138033</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1M 1%</t>
+          <t>ESD diode bidir 5.5V</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>R21, R26</t>
+          <t>D9</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>X1-SON-2 0.6x1.0mm</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
-        <is>
-          <t>C26083</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>ESD diode bidir 5.5V</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>D9</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>X1-SON-2 0.6x1.0mm</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
         <is>
           <t>C48260</t>
         </is>

</xml_diff>